<commit_message>
Yukti 0.3.0: self-contained server, desktop app, admin-only LLM config, HOD-only data, no invented data
- yukti-server.exe (PyInstaller) with bundled llama.cpp CUDA/Vulkan, model and pre-trained Laya; auto GPU backend
- Electron desktop client (plant-server or all-in-one mode launching the bundled server)
- Admin: users (CSV import, reset, disable), org AI settings, usage & health (measured only), feedback, backups/restore, model import, Laya benchmark
- Auth: forced password change, TOTP MFA with recovery codes
- Only HODs add/remove documents, only for their own department
- Findings workflow with per-role allowed actions; grey theme; Hindi/Kannada UI
- Removed invented data: 15 EXAMPLE documents (watermarked, badged), real MRPL departments, optimizer runs only on planner-entered model
- e2e suite: 74 checks
</commit_message>
<xml_diff>
--- a/data/corpus/contacts_oncall.xlsx
+++ b/data/corpus/contacts_oncall.xlsx
@@ -444,7 +444,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Yukti Refinery – Contacts   [SYNTHETIC – SIH DEMO]</t>
+          <t>Example Plant – Contacts   [EXAMPLE – prepared by Team UniMinds – NOT MRPL DATA]</t>
         </is>
       </c>
     </row>
@@ -1619,7 +1619,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Yukti Refinery – OnCall_2026-09-28   [SYNTHETIC – SIH DEMO]</t>
+          <t>Example Plant – OnCall_2026-09-28   [EXAMPLE – prepared by Team UniMinds – NOT MRPL DATA]</t>
         </is>
       </c>
     </row>

</xml_diff>